<commit_message>
Fix web E2E tests localhost/IPv6 binding issues by forcing 127.0.0.1
</commit_message>
<xml_diff>
--- a/sentinel-web/E2E_Test_Report_Sentinel.xlsx
+++ b/sentinel-web/E2E_Test_Report_Sentinel.xlsx
@@ -540,16 +540,16 @@
         <v>100</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>64.65000000000001</v>
+        <v>49.83</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16T06:03:24.633901Z</t>
+          <t>2026-06-16T06:20:14.937875Z</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16T06:04:29.286234Z</t>
+          <t>2026-06-16T06:21:04.769658Z</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.5</v>
+        <v>0.52</v>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>0.02</v>
+        <v>0.12</v>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>0.02</v>
+        <v>0.06</v>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
@@ -708,7 +708,7 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
@@ -800,7 +800,7 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>1.29</v>
+        <v>1.3</v>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>0.02</v>
+        <v>0.03</v>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
@@ -961,7 +961,7 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
@@ -984,7 +984,7 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>0.59</v>
+        <v>0.27</v>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
@@ -1007,7 +1007,7 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>0.75</v>
+        <v>0.4</v>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
@@ -1030,7 +1030,7 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>1.22</v>
+        <v>1.24</v>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
@@ -1053,7 +1053,7 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
@@ -1076,7 +1076,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>0.58</v>
+        <v>0.59</v>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
@@ -1122,7 +1122,7 @@
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>1.65</v>
+        <v>1.23</v>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
@@ -1145,7 +1145,7 @@
         </is>
       </c>
       <c r="D25" s="3" t="n">
-        <v>0.36</v>
+        <v>0.02</v>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
@@ -1168,7 +1168,7 @@
         </is>
       </c>
       <c r="D26" s="3" t="n">
-        <v>0.42</v>
+        <v>0.02</v>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
@@ -1191,7 +1191,7 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>0.11</v>
+        <v>0.02</v>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>0.04</v>
+        <v>0.02</v>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
@@ -1237,7 +1237,7 @@
         </is>
       </c>
       <c r="D29" s="3" t="n">
-        <v>0.04</v>
+        <v>0.02</v>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
@@ -1260,7 +1260,7 @@
         </is>
       </c>
       <c r="D30" s="3" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="D31" s="3" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
@@ -1306,7 +1306,7 @@
         </is>
       </c>
       <c r="D32" s="3" t="n">
-        <v>0.42</v>
+        <v>0.02</v>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
@@ -1329,7 +1329,7 @@
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>0.75</v>
+        <v>0.03</v>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
@@ -1352,7 +1352,7 @@
         </is>
       </c>
       <c r="D34" s="3" t="n">
-        <v>0.13</v>
+        <v>0.02</v>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
@@ -1375,7 +1375,7 @@
         </is>
       </c>
       <c r="D35" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.03</v>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
         </is>
       </c>
       <c r="D36" s="3" t="n">
-        <v>1.27</v>
+        <v>1.09</v>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
@@ -1421,7 +1421,7 @@
         </is>
       </c>
       <c r="D37" s="3" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
@@ -1444,7 +1444,7 @@
         </is>
       </c>
       <c r="D38" s="3" t="n">
-        <v>0.03</v>
+        <v>0.01</v>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
@@ -1467,7 +1467,7 @@
         </is>
       </c>
       <c r="D39" s="3" t="n">
-        <v>0.61</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
@@ -1490,7 +1490,7 @@
         </is>
       </c>
       <c r="D40" s="3" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
@@ -1513,7 +1513,7 @@
         </is>
       </c>
       <c r="D41" s="3" t="n">
-        <v>0.03</v>
+        <v>0.04</v>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
@@ -1582,7 +1582,7 @@
         </is>
       </c>
       <c r="D44" s="3" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
@@ -1605,7 +1605,7 @@
         </is>
       </c>
       <c r="D45" s="3" t="n">
-        <v>1.25</v>
+        <v>1.17</v>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
@@ -1628,7 +1628,7 @@
         </is>
       </c>
       <c r="D46" s="3" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
@@ -1651,7 +1651,7 @@
         </is>
       </c>
       <c r="D47" s="3" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
@@ -1697,7 +1697,7 @@
         </is>
       </c>
       <c r="D49" s="3" t="n">
-        <v>0.7</v>
+        <v>0.67</v>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
         </is>
       </c>
       <c r="D54" s="3" t="n">
-        <v>0.57</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
@@ -1904,7 +1904,7 @@
         </is>
       </c>
       <c r="D58" s="3" t="n">
-        <v>0.03</v>
+        <v>0.01</v>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
@@ -1927,7 +1927,7 @@
         </is>
       </c>
       <c r="D59" s="3" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
@@ -1950,7 +1950,7 @@
         </is>
       </c>
       <c r="D60" s="3" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
         </is>
       </c>
       <c r="D61" s="3" t="n">
-        <v>0.01</v>
+        <v>0.03</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
@@ -2019,7 +2019,7 @@
         </is>
       </c>
       <c r="D63" s="3" t="n">
-        <v>1.09</v>
+        <v>1.08</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
@@ -2042,7 +2042,7 @@
         </is>
       </c>
       <c r="D64" s="3" t="n">
-        <v>1.25</v>
+        <v>1.21</v>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
@@ -2065,7 +2065,7 @@
         </is>
       </c>
       <c r="D65" s="3" t="n">
-        <v>0.18</v>
+        <v>0.06</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
@@ -2111,7 +2111,7 @@
         </is>
       </c>
       <c r="D67" s="3" t="n">
-        <v>0.58</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
@@ -2180,7 +2180,7 @@
         </is>
       </c>
       <c r="D70" s="3" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
@@ -2249,7 +2249,7 @@
         </is>
       </c>
       <c r="D73" s="3" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
@@ -2272,7 +2272,7 @@
         </is>
       </c>
       <c r="D74" s="3" t="n">
-        <v>1.07</v>
+        <v>1.06</v>
       </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
@@ -2295,7 +2295,7 @@
         </is>
       </c>
       <c r="D75" s="3" t="n">
-        <v>3.02</v>
+        <v>3.06</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
@@ -2387,7 +2387,7 @@
         </is>
       </c>
       <c r="D79" s="3" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
@@ -2410,7 +2410,7 @@
         </is>
       </c>
       <c r="D80" s="3" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="E80" s="4" t="inlineStr">
         <is>
@@ -2479,7 +2479,7 @@
         </is>
       </c>
       <c r="D83" s="3" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="E83" s="4" t="inlineStr">
         <is>
@@ -2502,7 +2502,7 @@
         </is>
       </c>
       <c r="D84" s="3" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
@@ -2525,7 +2525,7 @@
         </is>
       </c>
       <c r="D85" s="3" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="E85" s="4" t="inlineStr">
         <is>
@@ -2571,7 +2571,7 @@
         </is>
       </c>
       <c r="D87" s="3" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="E87" s="4" t="inlineStr">
         <is>
@@ -2640,7 +2640,7 @@
         </is>
       </c>
       <c r="D90" s="3" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="E90" s="4" t="inlineStr">
         <is>
@@ -2801,7 +2801,7 @@
         </is>
       </c>
       <c r="D97" s="3" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="E97" s="4" t="inlineStr">
         <is>
@@ -2824,7 +2824,7 @@
         </is>
       </c>
       <c r="D98" s="3" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="E98" s="4" t="inlineStr">
         <is>
@@ -2916,7 +2916,7 @@
         </is>
       </c>
       <c r="D102" s="3" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="E102" s="4" t="inlineStr">
         <is>
@@ -2939,7 +2939,7 @@
         </is>
       </c>
       <c r="D103" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="E103" s="4" t="inlineStr">
         <is>
@@ -2985,7 +2985,7 @@
         </is>
       </c>
       <c r="D105" s="3" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="E105" s="4" t="inlineStr">
         <is>
@@ -3008,7 +3008,7 @@
         </is>
       </c>
       <c r="D106" s="3" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="E106" s="4" t="inlineStr">
         <is>
@@ -3077,7 +3077,7 @@
         </is>
       </c>
       <c r="D109" s="3" t="n">
-        <v>1.15</v>
+        <v>1.14</v>
       </c>
       <c r="E109" s="4" t="inlineStr">
         <is>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="D110" s="3" t="n">
-        <v>12.18</v>
+        <v>12.15</v>
       </c>
       <c r="E110" s="4" t="inlineStr">
         <is>
@@ -3123,7 +3123,7 @@
         </is>
       </c>
       <c r="D111" s="3" t="n">
-        <v>1.08</v>
+        <v>1.07</v>
       </c>
       <c r="E111" s="4" t="inlineStr">
         <is>
@@ -3247,7 +3247,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:43</t>
+          <t>2026-06-16 06:20:23</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -3257,14 +3257,14 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>[Authentication &amp; Redirection] test_001_login_page_renders → PASSED in 0.5s</t>
+          <t>[Authentication &amp; Redirection] test_001_login_page_renders → PASSED in 0.52s</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:43</t>
+          <t>2026-06-16 06:20:23</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -3281,7 +3281,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:43</t>
+          <t>2026-06-16 06:20:23</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -3291,14 +3291,14 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>[Authentication &amp; Redirection] test_003_login_subtitle → PASSED in 0.02s</t>
+          <t>[Authentication &amp; Redirection] test_003_login_subtitle → PASSED in 0.12s</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:43</t>
+          <t>2026-06-16 06:20:23</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -3308,14 +3308,14 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>[Authentication &amp; Redirection] test_004_login_email_input_exists → PASSED in 0.02s</t>
+          <t>[Authentication &amp; Redirection] test_004_login_email_input_exists → PASSED in 0.06s</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:43</t>
+          <t>2026-06-16 06:20:23</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -3325,14 +3325,14 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>[Authentication &amp; Redirection] test_005_login_submit_btn_exists → PASSED in 0.01s</t>
+          <t>[Authentication &amp; Redirection] test_005_login_submit_btn_exists → PASSED in 0.02s</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:43</t>
+          <t>2026-06-16 06:20:23</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -3349,7 +3349,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:43</t>
+          <t>2026-06-16 06:20:23</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -3366,7 +3366,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:44</t>
+          <t>2026-06-16 06:20:23</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -3383,7 +3383,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:45</t>
+          <t>2026-06-16 06:20:25</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -3393,14 +3393,14 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>[Authentication &amp; Redirection] test_009_login_invalid_email_displays_error → PASSED in 1.29s</t>
+          <t>[Authentication &amp; Redirection] test_009_login_invalid_email_displays_error → PASSED in 1.3s</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:45</t>
+          <t>2026-06-16 06:20:25</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -3410,14 +3410,14 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>[Authentication &amp; Redirection] test_010_register_page_renders → PASSED in 0.02s</t>
+          <t>[Authentication &amp; Redirection] test_010_register_page_renders → PASSED in 0.03s</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:45</t>
+          <t>2026-06-16 06:20:25</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -3434,7 +3434,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:45</t>
+          <t>2026-06-16 06:20:25</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -3451,7 +3451,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:45</t>
+          <t>2026-06-16 06:20:25</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -3468,7 +3468,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:45</t>
+          <t>2026-06-16 06:20:25</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -3485,7 +3485,7 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:45</t>
+          <t>2026-06-16 06:20:25</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -3502,7 +3502,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:45</t>
+          <t>2026-06-16 06:20:25</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -3512,14 +3512,14 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>[Authentication &amp; Redirection] test_016_register_login_link_exists → PASSED in 0.01s</t>
+          <t>[Authentication &amp; Redirection] test_016_register_login_link_exists → PASSED in 0.02s</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:46</t>
+          <t>2026-06-16 06:20:25</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -3529,14 +3529,14 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>[Authentication &amp; Redirection] test_017_register_duplicate_email_error → PASSED in 0.59s</t>
+          <t>[Authentication &amp; Redirection] test_017_register_duplicate_email_error → PASSED in 0.27s</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:46</t>
+          <t>2026-06-16 06:20:25</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -3546,14 +3546,14 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>[Authentication &amp; Redirection] test_018_register_success_flow → PASSED in 0.75s</t>
+          <t>[Authentication &amp; Redirection] test_018_register_success_flow → PASSED in 0.4s</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:47</t>
+          <t>2026-06-16 06:20:27</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -3563,14 +3563,14 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>[Admin Command Center] test_019_login_as_admin_redirects_dashboard → PASSED in 1.22s</t>
+          <t>[Admin Command Center] test_019_login_as_admin_redirects_dashboard → PASSED in 1.24s</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:49</t>
+          <t>2026-06-16 06:20:28</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -3580,14 +3580,14 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>[Authentication &amp; Redirection] test_020_login_as_user_redirects_portal → PASSED in 1.22s</t>
+          <t>[Authentication &amp; Redirection] test_020_login_as_user_redirects_portal → PASSED in 1.28s</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:49</t>
+          <t>2026-06-16 06:20:29</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -3597,14 +3597,14 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>[Safe Route Planner] test_021_route_protection_dashboard_direct → PASSED in 0.58s</t>
+          <t>[Safe Route Planner] test_021_route_protection_dashboard_direct → PASSED in 0.59s</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:50</t>
+          <t>2026-06-16 06:20:29</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -3621,7 +3621,7 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:51</t>
+          <t>2026-06-16 06:20:30</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -3631,14 +3631,14 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>[User Portal - Home &amp; SOS] test_023_portal_home_welcome_title → PASSED in 1.65s</t>
+          <t>[User Portal - Home &amp; SOS] test_023_portal_home_welcome_title → PASSED in 1.23s</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:52</t>
+          <t>2026-06-16 06:20:30</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -3648,14 +3648,14 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>[User Portal - Home &amp; SOS] test_024_portal_home_subtitle → PASSED in 0.36s</t>
+          <t>[User Portal - Home &amp; SOS] test_024_portal_home_subtitle → PASSED in 0.02s</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:52</t>
+          <t>2026-06-16 06:20:30</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -3665,14 +3665,14 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>[User Portal - Home &amp; SOS] test_025_portal_home_sos_btn_renders → PASSED in 0.42s</t>
+          <t>[User Portal - Home &amp; SOS] test_025_portal_home_sos_btn_renders → PASSED in 0.02s</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:52</t>
+          <t>2026-06-16 06:20:30</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -3682,14 +3682,14 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>[User Portal - Home &amp; SOS] test_026_portal_home_sos_initial_text → PASSED in 0.11s</t>
+          <t>[User Portal - Home &amp; SOS] test_026_portal_home_sos_initial_text → PASSED in 0.02s</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:52</t>
+          <t>2026-06-16 06:20:30</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -3699,14 +3699,14 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>[User Portal - Home &amp; SOS] test_027_portal_home_contacts_card_renders → PASSED in 0.04s</t>
+          <t>[User Portal - Home &amp; SOS] test_027_portal_home_contacts_card_renders → PASSED in 0.02s</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:52</t>
+          <t>2026-06-16 06:20:30</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -3716,14 +3716,14 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>[User Portal - Home &amp; SOS] test_028_portal_home_contacts_card_has_count → PASSED in 0.04s</t>
+          <t>[User Portal - Home &amp; SOS] test_028_portal_home_contacts_card_has_count → PASSED in 0.02s</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:52</t>
+          <t>2026-06-16 06:20:30</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -3733,14 +3733,14 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>[User Portal - Home &amp; SOS] test_029_portal_home_how_sos_works_card → PASSED in 0.05s</t>
+          <t>[User Portal - Home &amp; SOS] test_029_portal_home_how_sos_works_card → PASSED in 0.01s</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:52</t>
+          <t>2026-06-16 06:20:30</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -3750,14 +3750,14 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>[User Portal - Home &amp; SOS] test_030_portal_home_how_sos_works_steps → PASSED in 0.02s</t>
+          <t>[User Portal - Home &amp; SOS] test_030_portal_home_how_sos_works_steps → PASSED in 0.01s</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:53</t>
+          <t>2026-06-16 06:20:30</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -3767,14 +3767,14 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>[User Portal - Home &amp; SOS] test_031_portal_home_quick_actions_title → PASSED in 0.42s</t>
+          <t>[User Portal - Home &amp; SOS] test_031_portal_home_quick_actions_title → PASSED in 0.02s</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:54</t>
+          <t>2026-06-16 06:20:30</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -3784,14 +3784,14 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>[User Portal - Home &amp; SOS] test_032_portal_home_quick_action_contacts_link → PASSED in 0.75s</t>
+          <t>[User Portal - Home &amp; SOS] test_032_portal_home_quick_action_contacts_link → PASSED in 0.03s</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:54</t>
+          <t>2026-06-16 06:20:30</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -3801,14 +3801,14 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>[User Portal - Home &amp; SOS] test_033_portal_home_quick_action_report_link → PASSED in 0.13s</t>
+          <t>[User Portal - Home &amp; SOS] test_033_portal_home_quick_action_report_link → PASSED in 0.02s</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:54</t>
+          <t>2026-06-16 06:20:31</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -3818,14 +3818,14 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>[User Portal - Home &amp; SOS] test_034_portal_home_quick_action_route_link → PASSED in 0.07s</t>
+          <t>[User Portal - Home &amp; SOS] test_034_portal_home_quick_action_route_link → PASSED in 0.03s</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:55</t>
+          <t>2026-06-16 06:20:32</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -3835,14 +3835,14 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>[User Portal - Home &amp; SOS] test_035_portal_home_sos_trigger_flow → PASSED in 1.27s</t>
+          <t>[User Portal - Home &amp; SOS] test_035_portal_home_sos_trigger_flow → PASSED in 1.09s</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:55</t>
+          <t>2026-06-16 06:20:32</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -3852,14 +3852,14 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>[User Portal - Home &amp; SOS] test_036_portal_home_sos_coords_displayed → PASSED in 0.02s</t>
+          <t>[User Portal - Home &amp; SOS] test_036_portal_home_sos_coords_displayed → PASSED in 0.01s</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:55</t>
+          <t>2026-06-16 06:20:32</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -3869,14 +3869,14 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>[User Portal - Home &amp; SOS] test_037_portal_home_sos_btn_changes_to_sent → PASSED in 0.03s</t>
+          <t>[User Portal - Home &amp; SOS] test_037_portal_home_sos_btn_changes_to_sent → PASSED in 0.01s</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:56</t>
+          <t>2026-06-16 06:20:32</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -3886,14 +3886,14 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>[Trusted Contacts] test_038_portal_contacts_navigation → PASSED in 0.61s</t>
+          <t>[Trusted Contacts] test_038_portal_contacts_navigation → PASSED in 0.56s</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:56</t>
+          <t>2026-06-16 06:20:32</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -3903,14 +3903,14 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>[Trusted Contacts] test_039_portal_contacts_subtitle → PASSED in 0.02s</t>
+          <t>[Trusted Contacts] test_039_portal_contacts_subtitle → PASSED in 0.01s</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:56</t>
+          <t>2026-06-16 06:20:32</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -3920,14 +3920,14 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>[Trusted Contacts] test_040_portal_contacts_form_title → PASSED in 0.03s</t>
+          <t>[Trusted Contacts] test_040_portal_contacts_form_title → PASSED in 0.04s</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:56</t>
+          <t>2026-06-16 06:20:32</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -3944,7 +3944,7 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:56</t>
+          <t>2026-06-16 06:20:32</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -3961,7 +3961,7 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:56</t>
+          <t>2026-06-16 06:20:32</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -3971,14 +3971,14 @@
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>[Trusted Contacts] test_043_portal_contacts_submit_btn_exists → PASSED in 0.03s</t>
+          <t>[Trusted Contacts] test_043_portal_contacts_submit_btn_exists → PASSED in 0.02s</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:57</t>
+          <t>2026-06-16 06:20:33</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -3988,14 +3988,14 @@
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>[Trusted Contacts] test_044_portal_contacts_add_contact_success → PASSED in 1.25s</t>
+          <t>[Trusted Contacts] test_044_portal_contacts_add_contact_success → PASSED in 1.17s</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:57</t>
+          <t>2026-06-16 06:20:33</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -4005,14 +4005,14 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>[Trusted Contacts] test_045_portal_contacts_input_cleared_on_success → PASSED in 0.02s</t>
+          <t>[Trusted Contacts] test_045_portal_contacts_input_cleared_on_success → PASSED in 0.01s</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:57</t>
+          <t>2026-06-16 06:20:33</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -4022,14 +4022,14 @@
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>[Trusted Contacts] test_046_portal_contacts_initials_calculated_correctly → PASSED in 0.02s</t>
+          <t>[Trusted Contacts] test_046_portal_contacts_initials_calculated_correctly → PASSED in 0.01s</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:57</t>
+          <t>2026-06-16 06:20:34</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -4046,7 +4046,7 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:58</t>
+          <t>2026-06-16 06:20:34</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -4056,14 +4056,14 @@
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>[Trusted Contacts] test_048_portal_contacts_multiple_contacts_list → PASSED in 0.7s</t>
+          <t>[Trusted Contacts] test_048_portal_contacts_multiple_contacts_list → PASSED in 0.67s</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:58</t>
+          <t>2026-06-16 06:20:34</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -4080,7 +4080,7 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:58</t>
+          <t>2026-06-16 06:20:34</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -4097,7 +4097,7 @@
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:58</t>
+          <t>2026-06-16 06:20:34</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
@@ -4114,7 +4114,7 @@
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:58</t>
+          <t>2026-06-16 06:20:34</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
@@ -4131,7 +4131,7 @@
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:59</t>
+          <t>2026-06-16 06:20:34</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
@@ -4141,14 +4141,14 @@
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>[Report Incident] test_053_portal_report_navigation → PASSED in 0.57s</t>
+          <t>[Report Incident] test_053_portal_report_navigation → PASSED in 0.07s</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:59</t>
+          <t>2026-06-16 06:20:34</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
@@ -4165,7 +4165,7 @@
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:59</t>
+          <t>2026-06-16 06:20:34</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
@@ -4182,7 +4182,7 @@
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:59</t>
+          <t>2026-06-16 06:20:34</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
@@ -4199,7 +4199,7 @@
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:59</t>
+          <t>2026-06-16 06:20:34</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
@@ -4209,14 +4209,14 @@
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>[Report Incident] test_057_portal_report_severity_buttons → PASSED in 0.03s</t>
+          <t>[Report Incident] test_057_portal_report_severity_buttons → PASSED in 0.01s</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:59</t>
+          <t>2026-06-16 06:20:34</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
@@ -4226,14 +4226,14 @@
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>[Report Incident] test_058_portal_report_description_field → PASSED in 0.05s</t>
+          <t>[Report Incident] test_058_portal_report_description_field → PASSED in 0.01s</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:59</t>
+          <t>2026-06-16 06:20:34</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
@@ -4243,14 +4243,14 @@
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>[Report Incident] test_059_portal_report_use_mylocation_btn → PASSED in 0.01s</t>
+          <t>[Report Incident] test_059_portal_report_use_mylocation_btn → PASSED in 0.02s</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:59</t>
+          <t>2026-06-16 06:20:34</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
@@ -4260,14 +4260,14 @@
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>[Report Incident] test_060_portal_report_location_coordinates_text_initial → PASSED in 0.01s</t>
+          <t>[Report Incident] test_060_portal_report_location_coordinates_text_initial → PASSED in 0.03s</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:03:59</t>
+          <t>2026-06-16 06:20:34</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
@@ -4284,7 +4284,7 @@
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:00</t>
+          <t>2026-06-16 06:20:36</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
@@ -4294,14 +4294,14 @@
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>[Report Incident] test_062_portal_report_click_use_mylocation → PASSED in 1.09s</t>
+          <t>[Report Incident] test_062_portal_report_click_use_mylocation → PASSED in 1.08s</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:01</t>
+          <t>2026-06-16 06:20:37</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
@@ -4311,14 +4311,14 @@
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>[Report Incident] test_063_portal_report_submit_success_flow → PASSED in 1.25s</t>
+          <t>[Report Incident] test_063_portal_report_submit_success_flow → PASSED in 1.21s</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:01</t>
+          <t>2026-06-16 06:20:37</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
@@ -4328,14 +4328,14 @@
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>[Report Incident] test_064_portal_report_reset_form_flow → PASSED in 0.18s</t>
+          <t>[Report Incident] test_064_portal_report_reset_form_flow → PASSED in 0.06s</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:01</t>
+          <t>2026-06-16 06:20:37</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
@@ -4352,7 +4352,7 @@
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:02</t>
+          <t>2026-06-16 06:20:37</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
@@ -4362,14 +4362,14 @@
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>[Safe Route Planner] test_066_portal_route_navigation → PASSED in 0.58s</t>
+          <t>[Safe Route Planner] test_066_portal_route_navigation → PASSED in 0.56s</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:02</t>
+          <t>2026-06-16 06:20:37</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
@@ -4386,7 +4386,7 @@
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:02</t>
+          <t>2026-06-16 06:20:37</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
@@ -4403,7 +4403,7 @@
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:02</t>
+          <t>2026-06-16 06:20:37</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
@@ -4413,14 +4413,14 @@
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>[Safe Route Planner] test_069_portal_route_to_input_exists → PASSED in 0.01s</t>
+          <t>[Safe Route Planner] test_069_portal_route_to_input_exists → PASSED in 0.02s</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:02</t>
+          <t>2026-06-16 06:20:37</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
@@ -4437,7 +4437,7 @@
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:02</t>
+          <t>2026-06-16 06:20:37</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
@@ -4454,7 +4454,7 @@
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:02</t>
+          <t>2026-06-16 06:20:38</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
@@ -4464,14 +4464,14 @@
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>[Safe Route Planner] test_072_portal_route_map_container_exists → PASSED in 0.02s</t>
+          <t>[Safe Route Planner] test_072_portal_route_map_container_exists → PASSED in 0.01s</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:03</t>
+          <t>2026-06-16 06:20:39</t>
         </is>
       </c>
       <c r="B74" s="3" t="inlineStr">
@@ -4481,14 +4481,14 @@
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>[Safe Route Planner] test_073_portal_route_click_use_mylocation_fills_origin → PASSED in 1.07s</t>
+          <t>[Safe Route Planner] test_073_portal_route_click_use_mylocation_fills_origin → PASSED in 1.06s</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:06</t>
+          <t>2026-06-16 06:20:42</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
@@ -4498,14 +4498,14 @@
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>[Safe Route Planner] test_074_portal_route_empty_inputs_error_not_triggered_initially → PASSED in 3.02s</t>
+          <t>[Safe Route Planner] test_074_portal_route_empty_inputs_error_not_triggered_initially → PASSED in 3.06s</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:08</t>
+          <t>2026-06-16 06:20:44</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
@@ -4522,7 +4522,7 @@
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:09</t>
+          <t>2026-06-16 06:20:44</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
@@ -4539,7 +4539,7 @@
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:09</t>
+          <t>2026-06-16 06:20:44</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
@@ -4556,7 +4556,7 @@
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:09</t>
+          <t>2026-06-16 06:20:44</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
@@ -4566,14 +4566,14 @@
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>[User Profile] test_078_portal_profile_initials_circle → PASSED in 0.02s</t>
+          <t>[User Profile] test_078_portal_profile_initials_circle → PASSED in 0.01s</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:09</t>
+          <t>2026-06-16 06:20:44</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
@@ -4583,14 +4583,14 @@
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>[User Profile] test_079_portal_profile_display_name → PASSED in 0.02s</t>
+          <t>[User Profile] test_079_portal_profile_display_name → PASSED in 0.01s</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:09</t>
+          <t>2026-06-16 06:20:44</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
@@ -4607,7 +4607,7 @@
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:09</t>
+          <t>2026-06-16 06:20:44</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
@@ -4624,7 +4624,7 @@
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:09</t>
+          <t>2026-06-16 06:20:44</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
@@ -4634,14 +4634,14 @@
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>[Trusted Contacts] test_082_portal_profile_stats_contacts_count → PASSED in 0.02s</t>
+          <t>[Trusted Contacts] test_082_portal_profile_stats_contacts_count → PASSED in 0.01s</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:09</t>
+          <t>2026-06-16 06:20:44</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
@@ -4651,14 +4651,14 @@
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>[User Portal - Home &amp; SOS] test_083_portal_profile_stats_sos_count → PASSED in 0.02s</t>
+          <t>[User Portal - Home &amp; SOS] test_083_portal_profile_stats_sos_count → PASSED in 0.01s</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:09</t>
+          <t>2026-06-16 06:20:44</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
@@ -4668,14 +4668,14 @@
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>[User Profile] test_084_portal_profile_details_section → PASSED in 0.02s</t>
+          <t>[User Profile] test_084_portal_profile_details_section → PASSED in 0.01s</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:09</t>
+          <t>2026-06-16 06:20:44</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
@@ -4692,7 +4692,7 @@
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:09</t>
+          <t>2026-06-16 06:20:45</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
@@ -4702,14 +4702,14 @@
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>[User Profile] test_086_portal_profile_logout_btn_exists → PASSED in 0.02s</t>
+          <t>[User Profile] test_086_portal_profile_logout_btn_exists → PASSED in 0.01s</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:12</t>
+          <t>2026-06-16 06:20:47</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
@@ -4726,7 +4726,7 @@
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:12</t>
+          <t>2026-06-16 06:20:47</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
@@ -4743,7 +4743,7 @@
     <row r="90">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:12</t>
+          <t>2026-06-16 06:20:47</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
@@ -4753,14 +4753,14 @@
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>[Admin Command Center] test_089_admin_dashboard_subtitle → PASSED in 0.03s</t>
+          <t>[Admin Command Center] test_089_admin_dashboard_subtitle → PASSED in 0.02s</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:12</t>
+          <t>2026-06-16 06:20:47</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
@@ -4777,7 +4777,7 @@
     <row r="92">
       <c r="A92" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:12</t>
+          <t>2026-06-16 06:20:47</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
@@ -4794,7 +4794,7 @@
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:12</t>
+          <t>2026-06-16 06:20:47</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
@@ -4811,7 +4811,7 @@
     <row r="94">
       <c r="A94" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:12</t>
+          <t>2026-06-16 06:20:47</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
@@ -4828,7 +4828,7 @@
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:12</t>
+          <t>2026-06-16 06:20:47</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
@@ -4845,7 +4845,7 @@
     <row r="96">
       <c r="A96" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:12</t>
+          <t>2026-06-16 06:20:47</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
@@ -4862,7 +4862,7 @@
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:12</t>
+          <t>2026-06-16 06:20:47</t>
         </is>
       </c>
       <c r="B97" s="3" t="inlineStr">
@@ -4872,14 +4872,14 @@
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>[Trusted Contacts] test_096_admin_dashboard_stat_card_total_contacts → PASSED in 0.02s</t>
+          <t>[Trusted Contacts] test_096_admin_dashboard_stat_card_total_contacts → PASSED in 0.01s</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:12</t>
+          <t>2026-06-16 06:20:47</t>
         </is>
       </c>
       <c r="B98" s="3" t="inlineStr">
@@ -4889,14 +4889,14 @@
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>[Admin Command Center] test_097_admin_dashboard_hotspots_title → PASSED in 0.02s</t>
+          <t>[Admin Command Center] test_097_admin_dashboard_hotspots_title → PASSED in 0.01s</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:12</t>
+          <t>2026-06-16 06:20:47</t>
         </is>
       </c>
       <c r="B99" s="3" t="inlineStr">
@@ -4913,7 +4913,7 @@
     <row r="100">
       <c r="A100" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:12</t>
+          <t>2026-06-16 06:20:47</t>
         </is>
       </c>
       <c r="B100" s="3" t="inlineStr">
@@ -4930,7 +4930,7 @@
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:12</t>
+          <t>2026-06-16 06:20:47</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
@@ -4947,7 +4947,7 @@
     <row r="102">
       <c r="A102" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:12</t>
+          <t>2026-06-16 06:20:47</t>
         </is>
       </c>
       <c r="B102" s="3" t="inlineStr">
@@ -4957,14 +4957,14 @@
       </c>
       <c r="C102" s="4" t="inlineStr">
         <is>
-          <t>[Report Incident] test_101_admin_dashboard_reports_table_title → PASSED in 0.02s</t>
+          <t>[Report Incident] test_101_admin_dashboard_reports_table_title → PASSED in 0.01s</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:12</t>
+          <t>2026-06-16 06:20:48</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
@@ -4974,14 +4974,14 @@
       </c>
       <c r="C103" s="4" t="inlineStr">
         <is>
-          <t>[Report Incident] test_102_admin_dashboard_reports_table_headers → PASSED in 0.07s</t>
+          <t>[Report Incident] test_102_admin_dashboard_reports_table_headers → PASSED in 0.06s</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:12</t>
+          <t>2026-06-16 06:20:48</t>
         </is>
       </c>
       <c r="B104" s="3" t="inlineStr">
@@ -4998,7 +4998,7 @@
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:12</t>
+          <t>2026-06-16 06:20:48</t>
         </is>
       </c>
       <c r="B105" s="3" t="inlineStr">
@@ -5008,14 +5008,14 @@
       </c>
       <c r="C105" s="4" t="inlineStr">
         <is>
-          <t>[Admin Command Center] test_104_admin_dashboard_users_table_title → PASSED in 0.02s</t>
+          <t>[Admin Command Center] test_104_admin_dashboard_users_table_title → PASSED in 0.01s</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:12</t>
+          <t>2026-06-16 06:20:48</t>
         </is>
       </c>
       <c r="B106" s="3" t="inlineStr">
@@ -5025,14 +5025,14 @@
       </c>
       <c r="C106" s="4" t="inlineStr">
         <is>
-          <t>[Admin Command Center] test_105_admin_dashboard_users_table_data → PASSED in 0.02s</t>
+          <t>[Admin Command Center] test_105_admin_dashboard_users_table_data → PASSED in 0.01s</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:12</t>
+          <t>2026-06-16 06:20:48</t>
         </is>
       </c>
       <c r="B107" s="3" t="inlineStr">
@@ -5049,7 +5049,7 @@
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:12</t>
+          <t>2026-06-16 06:20:48</t>
         </is>
       </c>
       <c r="B108" s="3" t="inlineStr">
@@ -5066,7 +5066,7 @@
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:13</t>
+          <t>2026-06-16 06:20:49</t>
         </is>
       </c>
       <c r="B109" s="3" t="inlineStr">
@@ -5076,14 +5076,14 @@
       </c>
       <c r="C109" s="4" t="inlineStr">
         <is>
-          <t>[Admin Command Center] test_108_admin_dashboard_emergency_modal_details_flow → PASSED in 1.15s</t>
+          <t>[Admin Command Center] test_108_admin_dashboard_emergency_modal_details_flow → PASSED in 1.14s</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:25</t>
+          <t>2026-06-16 06:21:01</t>
         </is>
       </c>
       <c r="B110" s="3" t="inlineStr">
@@ -5093,14 +5093,14 @@
       </c>
       <c r="C110" s="4" t="inlineStr">
         <is>
-          <t>[User Portal - Home &amp; SOS] test_109_admin_dashboard_resolve_sos_flow → PASSED in 12.18s</t>
+          <t>[User Portal - Home &amp; SOS] test_109_admin_dashboard_resolve_sos_flow → PASSED in 12.15s</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:27</t>
+          <t>2026-06-16 06:21:02</t>
         </is>
       </c>
       <c r="B111" s="3" t="inlineStr">
@@ -5110,14 +5110,14 @@
       </c>
       <c r="C111" s="4" t="inlineStr">
         <is>
-          <t>[Admin Command Center] test_110_admin_logout_redirection → PASSED in 1.08s</t>
+          <t>[Admin Command Center] test_110_admin_logout_redirection → PASSED in 1.07s</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="3" t="inlineStr">
         <is>
-          <t>2026-06-16 06:04:27</t>
+          <t>2026-06-16 06:21:02</t>
         </is>
       </c>
       <c r="B112" s="3" t="inlineStr">

</xml_diff>